<commit_message>
DivPay repriced: constant adds at full adder cost, width envelope from 200k inputs; T6 3.06B (Google low-gate 2.99B, low-qubit 3.17B), strict 7.02B
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/technieken_analyse.xlsx
+++ b/docs/technieken_analyse.xlsx
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3631" uniqueCount="882">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3631" uniqueCount="883">
   <si>
     <t xml:space="preserve">Technieken-analyse ecdsa.fail (secp256k1 point add), 26-10-2026</t>
   </si>
@@ -2098,24 +2098,27 @@
     <t xml:space="preserve">Som railbreedte-envelop (535)</t>
   </si>
   <si>
-    <t xml:space="preserve">divsteps_sim.py envelop (1,500 invoeren, +4 bits marge)</t>
+    <t xml:space="preserve">width_check.py: envelop over 200,000 invoeren (som 72,197) + 2 bits marge per stap</t>
   </si>
   <si>
     <t xml:space="preserve">Som ceil(w/16) (535)</t>
   </si>
   <si>
-    <t xml:space="preserve">idem, voor de opgeknipte optellers</t>
+    <t xml:space="preserve">4,775 + 952/16 (benadering van de ruimere envelop)</t>
   </si>
   <si>
     <t xml:space="preserve">Som railbreedte-envelop (591)</t>
   </si>
   <si>
-    <t xml:space="preserve">idem</t>
+    <t xml:space="preserve">1,500-envelop + 2 + dezelfde verruiming (schatting)</t>
   </si>
   <si>
     <t xml:space="preserve">Railbreedte laatste stap</t>
   </si>
   <si>
+    <t xml:space="preserve">envelop + marge</t>
+  </si>
+  <si>
     <t xml:space="preserve">Blokgrootte opgeknipte opteller k</t>
   </si>
   <si>
@@ -2149,10 +2152,10 @@
     <t xml:space="preserve">Component (Toffoli)</t>
   </si>
   <si>
-    <t xml:space="preserve">T6 (generiek, 2.95B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strikt (geen enkele leader-techniek)</t>
+    <t xml:space="preserve">T6 (generieke primitieven)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strikt (geen leader-constructie)</t>
   </si>
   <si>
     <t xml:space="preserve">Opteller n bits (T)</t>
@@ -2209,7 +2212,7 @@
     <t xml:space="preserve">Score (T x Q)</t>
   </si>
   <si>
-    <t xml:space="preserve">T6 gebruikt generieke primitieven die de leader óók gebruikt (venster-vergelijkers #G17, opgeknipte optellers #G19, Solinas #G24, meting-uncompute #G14). Strikt vermijdt alle technieken met 'In leader' = ja/deels.</t>
+    <t xml:space="preserve">T6 gebruikt generieke primitieven die de leader óók gebruikt (venster-vergelijkers #G17, opgeknipte optellers #G19, Solinas #G24, meting-uncompute #G14). Strikt = geen van de leader-constructies uit blad Gebruikt (G-ids); elementaire poorten, optellers en vergelijkers deelt elk circuit en blijven toegestaan.</t>
   </si>
   <si>
     <t xml:space="preserve">Vergelijking: score = gemiddeld uitgevoerde Toffoli x piek-qubits</t>
@@ -2305,7 +2308,7 @@
     <t xml:space="preserve">Ontwerp-blad (kostenmodel, niet gebouwd)</t>
   </si>
   <si>
-    <t xml:space="preserve">Nieuw: DivPay strikt (geen leader-techniek)</t>
+    <t xml:space="preserve">Nieuw: DivPay strikt (geen leader-constructie)</t>
   </si>
   <si>
     <t xml:space="preserve">ja (bewezen 591 stappen)</t>
@@ -41905,7 +41908,7 @@
         <v>681</v>
       </c>
       <c r="B7" s="9" t="n">
-        <v>72315</v>
+        <v>73267</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>682</v>
@@ -41916,7 +41919,7 @@
         <v>683</v>
       </c>
       <c r="B8" s="9" t="n">
-        <v>4775</v>
+        <v>4835</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>684</v>
@@ -41927,7 +41930,7 @@
         <v>685</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>72651</v>
+        <v>73603</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>686</v>
@@ -41938,65 +41941,65 @@
         <v>687</v>
       </c>
       <c r="B10" s="9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>16</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B12" s="9" t="n">
         <v>40</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B13" s="9" t="n">
         <v>42</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B14" s="9" t="n">
         <v>1.58823529411765</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B15" s="9" t="n">
         <v>4</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -42006,18 +42009,18 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B18" s="11" t="n">
         <f aca="false">$B$4-1+2*ROUNDUP($B$4/$B$11,0)</f>
@@ -42030,20 +42033,20 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B19" s="11" t="n">
         <f aca="false">2*$B$7-$B$5+2*$B$8+$B$5*$B$13</f>
-        <v>176115</v>
+        <v>178139</v>
       </c>
       <c r="C19" s="11" t="n">
         <f aca="false">3*$B$9-$B$6+$B$6*$B$13</f>
-        <v>242184</v>
+        <v>245040</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B20" s="11" t="n">
         <f aca="false">$B$4</f>
@@ -42056,7 +42059,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B21" s="11" t="n">
         <f aca="false">B18</f>
@@ -42069,59 +42072,59 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B22" s="11" t="n">
-        <f aca="false">4*$B$12+$B$4</f>
-        <v>416</v>
+        <f aca="false">4*$B$12+B18</f>
+        <v>447</v>
       </c>
       <c r="C22" s="11" t="n">
-        <f aca="false">5*$B$4</f>
-        <v>1280</v>
+        <f aca="false">4*$B$4+C18</f>
+        <v>1535</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B23" s="11" t="n">
-        <f aca="false">$B$4+$B$12</f>
-        <v>296</v>
+        <f aca="false">B18+$B$12</f>
+        <v>327</v>
       </c>
       <c r="C23" s="11" t="n">
-        <f aca="false">2*$B$4</f>
-        <v>512</v>
+        <f aca="false">C18+$B$4</f>
+        <v>767</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B24" s="11" t="n">
         <f aca="false">$B$5*(B20+B21+B22+B23)</f>
-        <v>671425</v>
+        <v>704595</v>
       </c>
       <c r="C24" s="11" t="n">
         <f aca="false">$B$6*(C20+C21+C22+C23)</f>
-        <v>1512369</v>
+        <v>1813779</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B25" s="11" t="n">
         <f aca="false">2*B19+B24</f>
-        <v>1023655</v>
+        <v>1060873</v>
       </c>
       <c r="C25" s="11" t="n">
         <f aca="false">2*C19+C24</f>
-        <v>1996737</v>
+        <v>2303859</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B26" s="11" t="n">
         <f aca="false">$B$4^2/2+18*$B$4+B18</f>
@@ -42134,7 +42137,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B27" s="11" t="n">
         <f aca="false">4*$B$4</f>
@@ -42147,20 +42150,20 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B28" s="11" t="n">
         <f aca="false">2*B25+B26+B27</f>
-        <v>2085997</v>
+        <v>2160433</v>
       </c>
       <c r="C28" s="11" t="n">
         <f aca="false">2*C25+C26+C27</f>
-        <v>4093313</v>
+        <v>4707557</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B29" s="11" t="n">
         <f aca="false">ROUNDUP($B$5*$B$14,0)</f>
@@ -42173,7 +42176,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B30" s="11" t="n">
         <f aca="false">2*$B$4</f>
@@ -42186,20 +42189,20 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">2*$B$10+11+8</f>
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C31" s="11" t="n">
         <f aca="false">2*$B$10+11+8</f>
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B32" s="11" t="n">
         <f aca="false">$B$11+1</f>
@@ -42212,7 +42215,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B33" s="11" t="n">
         <f aca="false">$B$15</f>
@@ -42225,28 +42228,28 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B34" s="11" t="n">
         <f aca="false">SUM(B29:B33)</f>
-        <v>1414</v>
+        <v>1418</v>
       </c>
       <c r="C34" s="11" t="n">
         <f aca="false">SUM(C29:C33)</f>
-        <v>1487</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B35" s="11" t="n">
         <f aca="false">B28*B34</f>
-        <v>2949599758</v>
+        <v>3063493994</v>
       </c>
       <c r="C35" s="11" t="n">
         <f aca="false">C28*C34</f>
-        <v>6086756431</v>
+        <v>7018967487</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -42256,7 +42259,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -42292,7 +42295,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -42314,25 +42317,25 @@
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>25</v>
@@ -42340,7 +42343,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B4" s="12" t="n">
         <v>741645</v>
@@ -42361,15 +42364,15 @@
         <v>0.305827879699248</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>784645</v>
@@ -42390,15 +42393,15 @@
         <v>0.325919376775272</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>2100000</v>
@@ -42419,15 +42422,15 @@
         <v>1</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>2700000</v>
@@ -42448,15 +42451,15 @@
         <v>1.06015037593985</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B8" s="12" t="n">
         <v>1356000</v>
@@ -42477,15 +42480,15 @@
         <v>0.642995488721805</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B9" s="12" t="n">
         <v>2218127</v>
@@ -42506,15 +42509,15 @@
         <v>0.661917263492064</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B10" s="12" t="n">
         <v>2390000</v>
@@ -42535,15 +42538,15 @@
         <v>0.952006683375104</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B11" s="12" t="n">
         <v>3942753</v>
@@ -42567,69 +42570,69 @@
         <v>73</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B12" s="15" t="n">
         <f aca="false">Ontwerp!B28</f>
-        <v>2085997</v>
+        <v>2160433</v>
       </c>
       <c r="C12" s="15" t="n">
         <f aca="false">Ontwerp!B34</f>
-        <v>1414</v>
+        <v>1418</v>
       </c>
       <c r="D12" s="11" t="n">
         <f aca="false">B12*C12</f>
-        <v>2949599758</v>
+        <v>3063493994</v>
       </c>
       <c r="E12" s="13" t="n">
         <f aca="false">D12/$D$4</f>
-        <v>3.22293729564966</v>
+        <v>3.34738603821832</v>
       </c>
       <c r="F12" s="14" t="n">
         <f aca="false">D12/$D$6</f>
-        <v>0.985664079532164</v>
+        <v>1.02372397460317</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B13" s="15" t="n">
         <f aca="false">Ontwerp!C28</f>
-        <v>4093313</v>
+        <v>4707557</v>
       </c>
       <c r="C13" s="15" t="n">
         <f aca="false">Ontwerp!C34</f>
-        <v>1487</v>
+        <v>1491</v>
       </c>
       <c r="D13" s="11" t="n">
         <f aca="false">B13*C13</f>
-        <v>6086756431</v>
+        <v>7018967487</v>
       </c>
       <c r="E13" s="13" t="n">
         <f aca="false">D13/$D$4</f>
-        <v>6.65081228658187</v>
+        <v>7.66941074952606</v>
       </c>
       <c r="F13" s="14" t="n">
         <f aca="false">D13/$D$6</f>
-        <v>2.03400381988304</v>
+        <v>2.34551962807018</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -42644,11 +42647,11 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B15" s="2" t="str">
         <f aca="false">IF(D12&lt;D6,"ja, met "&amp;ROUND((1-D12/D6)*100,1)&amp;" procent","nee")</f>
-        <v>ja, met 1,4 procent</v>
+        <v>nee</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -42659,11 +42662,11 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B16" s="2" t="str">
         <f aca="false">IF(D13&lt;D6,"ja","nee, "&amp;ROUND(D13/D6,2)&amp;"x zo hoog")</f>
-        <v>nee, 2,03x zo hoog</v>
+        <v>nee, 2,35x zo hoog</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -42698,7 +42701,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -42726,48 +42729,48 @@
     </row>
     <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="D4" s="9" t="n">
         <v>10698739917</v>
@@ -42788,21 +42791,21 @@
         <v>3904012</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>10572302800</v>
@@ -42823,21 +42826,21 @@
         <v>3839944</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>10318536120</v>
@@ -42858,7 +42861,7 @@
         <v>3546654</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K6" s="9" t="s">
         <v>85</v>
@@ -42866,13 +42869,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>9591294596</v>
@@ -42893,21 +42896,21 @@
         <v>3656039</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="D8" s="9" t="n">
         <v>8367457560</v>
@@ -42928,21 +42931,21 @@
         <v>3361759</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>7754110980</v>
@@ -42963,21 +42966,21 @@
         <v>3063680</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>7074763080</v>
@@ -42998,21 +43001,21 @@
         <v>3015004</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="D11" s="9" t="n">
         <v>6961644236</v>
@@ -43033,21 +43036,21 @@
         <v>2973304</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="D12" s="9" t="n">
         <v>6865358936</v>
@@ -43068,21 +43071,21 @@
         <v>2929804</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>6764917436</v>
@@ -43103,21 +43106,21 @@
         <v>2870041</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="D14" s="9" t="n">
         <v>6453615747</v>
@@ -43138,21 +43141,21 @@
         <v>2615899</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="D15" s="9" t="n">
         <v>5882154410</v>
@@ -43173,21 +43176,21 @@
         <v>2462914</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D16" s="9" t="n">
         <v>5547081566</v>
@@ -43208,21 +43211,21 @@
         <v>2560503</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D17" s="9" t="n">
         <v>5120690122</v>
@@ -43243,21 +43246,21 @@
         <v>2447846</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D18" s="9" t="n">
         <v>4068676284</v>
@@ -43278,21 +43281,21 @@
         <v>2223350</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D19" s="9" t="n">
         <v>3775248300</v>
@@ -43313,21 +43316,21 @@
         <v>2083878</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D20" s="9" t="n">
         <v>3538424844</v>
@@ -43348,21 +43351,21 @@
         <v>1981734</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D21" s="9" t="n">
         <v>3364984332</v>
@@ -43383,21 +43386,21 @@
         <v>1952382</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D22" s="9" t="n">
         <v>3315144636</v>
@@ -43418,21 +43421,21 @@
         <v>1928442</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>3270229140</v>
@@ -43453,21 +43456,21 @@
         <v>1861990</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D24" s="9" t="n">
         <v>3161659020</v>
@@ -43488,21 +43491,21 @@
         <v>1838050</v>
       </c>
       <c r="J24" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K24" s="9" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D25" s="9" t="n">
         <v>3121008900</v>
@@ -43523,21 +43526,21 @@
         <v>1704086</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D26" s="9" t="n">
         <v>2822498802</v>
@@ -43558,21 +43561,21 @@
         <v>1770897</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D27" s="9" t="n">
         <v>2731939151</v>
@@ -43593,21 +43596,21 @@
         <v>1689505</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D28" s="9" t="n">
         <v>2574991500</v>
@@ -43628,21 +43631,21 @@
         <v>1732283</v>
       </c>
       <c r="J28" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="D29" s="9" t="n">
         <v>2379298050</v>
@@ -43663,21 +43666,21 @@
         <v>1629451</v>
       </c>
       <c r="J29" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K29" s="9" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>2257725570</v>
@@ -43698,21 +43701,21 @@
         <v>1602999</v>
       </c>
       <c r="J30" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K30" s="9" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="D31" s="9" t="n">
         <v>2221196370</v>
@@ -43733,21 +43736,21 @@
         <v>1579823</v>
       </c>
       <c r="J31" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K31" s="9" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="D32" s="9" t="n">
         <v>2195953970</v>
@@ -43768,21 +43771,21 @@
         <v>1551423</v>
       </c>
       <c r="J32" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K32" s="9" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="D33" s="9" t="n">
         <v>2089123794</v>
@@ -43803,21 +43806,21 @@
         <v>1565417</v>
       </c>
       <c r="J33" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K33" s="9" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="D34" s="9" t="n">
         <v>1891349200</v>
@@ -43838,21 +43841,21 @@
         <v>1404058</v>
       </c>
       <c r="J34" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K34" s="9" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="D35" s="9" t="n">
         <v>1820641701</v>
@@ -43873,21 +43876,21 @@
         <v>1386820</v>
       </c>
       <c r="J35" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K35" s="9" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="D36" s="9" t="n">
         <v>1743174081</v>
@@ -43908,21 +43911,21 @@
         <v>1405548</v>
       </c>
       <c r="J36" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K36" s="9" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="D37" s="9" t="n">
         <v>1641521688</v>
@@ -43943,21 +43946,21 @@
         <v>1391013</v>
       </c>
       <c r="J37" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K37" s="9" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="D38" s="9" t="n">
         <v>1571592960</v>
@@ -43978,21 +43981,21 @@
         <v>1320763</v>
       </c>
       <c r="J38" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K38" s="9" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="D39" s="9" t="n">
         <v>1477492400</v>
@@ -44013,21 +44016,21 @@
         <v>952707</v>
       </c>
       <c r="J39" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K39" s="9" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="D40" s="9" t="n">
         <v>1237028156</v>
@@ -44048,21 +44051,21 @@
         <v>939902</v>
       </c>
       <c r="J40" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K40" s="9" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="D41" s="9" t="n">
         <v>1137367864</v>
@@ -44083,21 +44086,21 @@
         <v>897597</v>
       </c>
       <c r="J41" s="9" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="K41" s="9" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="D42" s="9" t="n">
         <v>1107467010</v>
@@ -44118,21 +44121,21 @@
         <v>804160</v>
       </c>
       <c r="J42" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K42" s="9" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="9" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="D43" s="9" t="n">
         <v>983732808</v>
@@ -44153,21 +44156,21 @@
         <v>786948</v>
       </c>
       <c r="J43" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K43" s="9" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="9" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>971373636</v>
@@ -44188,10 +44191,10 @@
         <v>774510</v>
       </c>
       <c r="J44" s="9" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="K44" s="9" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
     </row>
   </sheetData>

</xml_diff>